<commit_message>
Final commit before migrating to company repo
</commit_message>
<xml_diff>
--- a/EPTS Test Cases/API Test Cases/Change Password.xlsx
+++ b/EPTS Test Cases/API Test Cases/Change Password.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srinivas\Desktop\MogoMantra Project\EPTS Testing\EPTS Test Cases\API Test Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230AE29C-F344-4368-9EB7-04D8D32C59DE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B901F244-EA0F-471F-9D6D-619587EA5729}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="53">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -190,6 +190,15 @@
   </si>
   <si>
     <t>Verify with Same password (New &amp; Confirm)</t>
+  </si>
+  <si>
+    <t>1st Retest Result</t>
+  </si>
+  <si>
+    <t>New password cannot be the same as the old password</t>
+  </si>
+  <si>
+    <t>401 Bad Request</t>
   </si>
 </sst>
 </file>
@@ -327,10 +336,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="10" customWidth="1"/>
@@ -625,48 +634,70 @@
     <col min="6" max="7" width="16.5703125" style="10" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" style="10" customWidth="1"/>
     <col min="9" max="9" width="12.5703125" style="10" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="10"/>
+    <col min="10" max="10" width="9.140625" style="10"/>
+    <col min="11" max="11" width="15.140625" style="10" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="H1" s="11" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-    </row>
-    <row r="2" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-    </row>
-    <row r="3" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-    </row>
-    <row r="4" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-    </row>
-    <row r="5" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-    </row>
-    <row r="6" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
-    </row>
-    <row r="7" spans="1:10" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+    </row>
+    <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -697,8 +728,17 @@
       <c r="J7" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>19</v>
       </c>
@@ -729,8 +769,17 @@
       <c r="J8" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
@@ -761,8 +810,17 @@
       <c r="J9" s="4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>21</v>
       </c>
@@ -793,8 +851,17 @@
       <c r="J10" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K10" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>22</v>
       </c>
@@ -825,8 +892,17 @@
       <c r="J11" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>23</v>
       </c>
@@ -857,8 +933,17 @@
       <c r="J12" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K12" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>24</v>
       </c>
@@ -889,8 +974,17 @@
       <c r="J13" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" s="10" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>25</v>
       </c>
@@ -921,10 +1015,20 @@
       <c r="J14" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="K14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="H1:J6"/>
+    <mergeCell ref="K1:M6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -935,7 +1039,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$C$3:$C$5</xm:f>
           </x14:formula1>
-          <xm:sqref>J8:J14</xm:sqref>
+          <xm:sqref>J8:J14 M8:M14</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>